<commit_message>
add plot extractions from sharp 2020
</commit_message>
<xml_diff>
--- a/Misc/Sharp_calculated.xlsx
+++ b/Misc/Sharp_calculated.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brookesienkiewicz/Documents/Code_notebook/Misc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C4357B1C-DE1F-0F4D-88FE-F0C0D17329BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{645A4585-D367-9440-BD77-46E1033EAA23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{3432E517-2846-BE4F-B9C3-C79612C8F25C}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="15080" windowHeight="18900" xr2:uid="{3432E517-2846-BE4F-B9C3-C79612C8F25C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="72">
   <si>
     <t>Location</t>
   </si>
@@ -221,9 +221,6 @@
     <t>Bar53</t>
   </si>
   <si>
-    <t>D_calculated</t>
-  </si>
-  <si>
     <t>Bar6</t>
   </si>
   <si>
@@ -249,6 +246,12 @@
   </si>
   <si>
     <t>Dead_Calculated</t>
+  </si>
+  <si>
+    <t>Dis_calculated</t>
+  </si>
+  <si>
+    <t>check</t>
   </si>
 </sst>
 </file>
@@ -621,13 +624,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6B9ADA7-011A-D64A-B347-6E134C209E83}">
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="7" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -647,13 +650,16 @@
         <v>3</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+        <v>69</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -670,8 +676,12 @@
         <f>100-(G2+D2)</f>
         <v>4.6600708905998545E-2</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I2" s="1">
+        <f>SUM(D2,G2,H2)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -688,8 +698,12 @@
         <f t="shared" ref="H3:H57" si="0">100-(G3+D3)</f>
         <v>0.11857372266079835</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I3" s="1">
+        <f t="shared" ref="I3:I56" si="1">SUM(D3,G3,H3)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -716,8 +730,12 @@
         <f t="shared" si="0"/>
         <v>1.9944037144895788E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I4" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -737,15 +755,19 @@
         <v>99.793459260527698</v>
       </c>
       <c r="G5" s="1">
-        <f t="shared" ref="G3:G29" si="1">F5-D5</f>
+        <f t="shared" ref="G5:G28" si="2">F5-D5</f>
         <v>1.2928485804110039</v>
       </c>
       <c r="H5" s="1">
         <f t="shared" si="0"/>
         <v>0.20654073947230245</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I5" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -765,15 +787,19 @@
         <v>99.769468255942797</v>
       </c>
       <c r="G6" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.9419385377926943</v>
       </c>
       <c r="H6" s="1">
         <f t="shared" si="0"/>
         <v>0.23053174405720256</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I6" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -793,15 +819,19 @@
         <v>99.153699138262496</v>
       </c>
       <c r="G7" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.1984258023658896</v>
       </c>
       <c r="H7" s="1">
         <f t="shared" si="0"/>
         <v>0.84630086173750385</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I7" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -809,7 +839,7 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D8" s="1">
         <v>89.817644131816394</v>
@@ -821,15 +851,19 @@
         <v>97.830028781127695</v>
       </c>
       <c r="G8" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8.0123846493113007</v>
       </c>
       <c r="H8" s="1">
         <f t="shared" si="0"/>
         <v>2.1699712188723055</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I8" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -849,15 +883,19 @@
         <v>95.455085931416406</v>
       </c>
       <c r="G9" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>11.249115483164303</v>
       </c>
       <c r="H9" s="1">
         <f t="shared" si="0"/>
         <v>4.5449140685835943</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I9" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -877,15 +915,19 @@
         <v>93.182604663786606</v>
       </c>
       <c r="G10" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14.741139483862199</v>
       </c>
       <c r="H10" s="1">
         <f t="shared" si="0"/>
         <v>6.8173953362133943</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I10" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>1</v>
       </c>
@@ -905,15 +947,19 @@
         <v>91.528113903150597</v>
       </c>
       <c r="G11" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>20.657143503365191</v>
       </c>
       <c r="H11" s="1">
         <f t="shared" si="0"/>
         <v>8.4718860968494027</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I11" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -933,15 +979,19 @@
         <v>85.718736570691803</v>
       </c>
       <c r="G12" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>22.491566798388305</v>
       </c>
       <c r="H12" s="1">
         <f t="shared" si="0"/>
         <v>14.281263429308197</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I12" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>1</v>
       </c>
@@ -961,15 +1011,19 @@
         <v>81.333714065998606</v>
       </c>
       <c r="G13" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>31.068350937507006</v>
       </c>
       <c r="H13" s="1">
         <f t="shared" si="0"/>
         <v>18.666285934001394</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I13" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>1</v>
       </c>
@@ -989,15 +1043,19 @@
         <v>80.288772532965396</v>
       </c>
       <c r="G14" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>35.639970144527695</v>
       </c>
       <c r="H14" s="1">
         <f t="shared" si="0"/>
         <v>19.711227467034604</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I14" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>1</v>
       </c>
@@ -1017,15 +1075,19 @@
         <v>80.487364737585196</v>
       </c>
       <c r="G15" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>36.359700282075998</v>
       </c>
       <c r="H15" s="1">
         <f t="shared" si="0"/>
         <v>19.512635262414804</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I15" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>1</v>
       </c>
@@ -1045,15 +1107,19 @@
         <v>80.4007305543618</v>
       </c>
       <c r="G16" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>36.572953656164501</v>
       </c>
       <c r="H16" s="1">
         <f t="shared" si="0"/>
         <v>19.5992694456382</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I16" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>1</v>
       </c>
@@ -1073,15 +1139,19 @@
         <v>80.201694071879302</v>
       </c>
       <c r="G17" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>36.355257503449202</v>
       </c>
       <c r="H17" s="1">
         <f t="shared" si="0"/>
         <v>19.798305928120698</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I17" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>1</v>
       </c>
@@ -1101,15 +1171,19 @@
         <v>80.027537149707101</v>
       </c>
       <c r="G18" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>36.1930960835695</v>
       </c>
       <c r="H18" s="1">
         <f t="shared" si="0"/>
         <v>19.972462850292899</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I18" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>1</v>
       </c>
@@ -1129,15 +1203,19 @@
         <v>79.927574630603104</v>
       </c>
       <c r="G19" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>36.286394434733104</v>
       </c>
       <c r="H19" s="1">
         <f t="shared" si="0"/>
         <v>20.072425369396896</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I19" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>1</v>
       </c>
@@ -1157,15 +1235,19 @@
         <v>80.0208729817668</v>
       </c>
       <c r="G20" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>36.293058602673398</v>
       </c>
       <c r="H20" s="1">
         <f t="shared" si="0"/>
         <v>19.9791270182332</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I20" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>1</v>
       </c>
@@ -1185,15 +1267,19 @@
         <v>80.027537149707101</v>
       </c>
       <c r="G21" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>36.386356953837101</v>
       </c>
       <c r="H21" s="1">
         <f t="shared" si="0"/>
         <v>19.972462850292899</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I21" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>1</v>
       </c>
@@ -1213,15 +1299,19 @@
         <v>79.596032275574998</v>
       </c>
       <c r="G22" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>36.275565161830201</v>
       </c>
       <c r="H22" s="1">
         <f t="shared" si="0"/>
         <v>20.403967724425002</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I22" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>1</v>
       </c>
@@ -1241,15 +1331,19 @@
         <v>79.407769531262602</v>
       </c>
       <c r="G23" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>36.239745259151299</v>
       </c>
       <c r="H23" s="1">
         <f t="shared" si="0"/>
         <v>20.592230468737398</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I23" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>1</v>
       </c>
@@ -1269,15 +1363,19 @@
         <v>79.001255286906499</v>
       </c>
       <c r="G24" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>37.226042114310196</v>
       </c>
       <c r="H24" s="1">
         <f t="shared" si="0"/>
         <v>20.998744713093501</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I24" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>1</v>
       </c>
@@ -1297,15 +1395,19 @@
         <v>79.274930450319999</v>
       </c>
       <c r="G25" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>37.512157057878902</v>
       </c>
       <c r="H25" s="1">
         <f t="shared" si="0"/>
         <v>20.725069549680001</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I25" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>1</v>
       </c>
@@ -1325,15 +1427,19 @@
         <v>78.907956935742803</v>
       </c>
       <c r="G26" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>37.3193404654739</v>
       </c>
       <c r="H26" s="1">
         <f t="shared" si="0"/>
         <v>21.092043064257197</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I26" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>1</v>
       </c>
@@ -1353,15 +1459,19 @@
         <v>78.441465179924407</v>
       </c>
       <c r="G27" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>37.985757259500303</v>
       </c>
       <c r="H27" s="1">
         <f t="shared" si="0"/>
         <v>21.558534820075593</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I27" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>1</v>
       </c>
@@ -1381,15 +1491,19 @@
         <v>78.435245289846804</v>
       </c>
       <c r="G28" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>39.023590346730607</v>
       </c>
       <c r="H28" s="1">
         <f t="shared" si="0"/>
         <v>21.564754710153196</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I28" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>1</v>
       </c>
@@ -1416,8 +1530,12 @@
         <f t="shared" si="0"/>
         <v>21.931728224730307</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I29" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -1435,8 +1553,12 @@
         <f t="shared" si="0"/>
         <v>0.28651075475539756</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I30" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -1454,8 +1576,12 @@
         <f t="shared" si="0"/>
         <v>0.29317492269569811</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I31" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>4</v>
       </c>
@@ -1475,15 +1601,19 @@
         <v>99.483353312374106</v>
       </c>
       <c r="G32" s="1">
-        <f t="shared" ref="G30:G57" si="2">F32-D32</f>
+        <f t="shared" ref="G32:G56" si="3">F32-D32</f>
         <v>2.1089870141619116</v>
       </c>
       <c r="H32" s="1">
         <f t="shared" si="0"/>
         <v>0.51664668762589372</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I32" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>4</v>
       </c>
@@ -1503,15 +1633,19 @@
         <v>99.793459260527698</v>
       </c>
       <c r="G33" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.2258320920478951</v>
       </c>
       <c r="H33" s="1">
         <f t="shared" si="0"/>
         <v>0.20654073947230245</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I33" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>4</v>
       </c>
@@ -1531,15 +1665,19 @@
         <v>99.7756881460204</v>
       </c>
       <c r="G34" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.4013218478082052</v>
       </c>
       <c r="H34" s="1">
         <f t="shared" si="0"/>
         <v>0.22431185397960007</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I34" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>4</v>
       </c>
@@ -1559,15 +1697,19 @@
         <v>99</v>
       </c>
       <c r="G35" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.1117431524665022</v>
       </c>
       <c r="H35" s="1">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I35" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>4</v>
       </c>
@@ -1587,15 +1729,19 @@
         <v>98.873804084771393</v>
       </c>
       <c r="G36" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5.6041209598986939</v>
       </c>
       <c r="H36" s="1">
         <f t="shared" si="0"/>
         <v>1.1261959152286067</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I36" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>4</v>
       </c>
@@ -1615,15 +1761,19 @@
         <v>98.307794087711699</v>
       </c>
       <c r="G37" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>7.7748625969737049</v>
       </c>
       <c r="H37" s="1">
         <f t="shared" si="0"/>
         <v>1.6922059122883013</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I37" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>4</v>
       </c>
@@ -1643,15 +1793,19 @@
         <v>97.567627168479802</v>
       </c>
       <c r="G38" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>11.575659712237197</v>
       </c>
       <c r="H38" s="1">
         <f t="shared" si="0"/>
         <v>2.4323728315201976</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I38" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>4</v>
       </c>
@@ -1671,15 +1825,19 @@
         <v>96.168151901024501</v>
       </c>
       <c r="G39" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>16.707069026239807</v>
       </c>
       <c r="H39" s="1">
         <f t="shared" si="0"/>
         <v>3.8318480989754988</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I39" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>4</v>
       </c>
@@ -1699,15 +1857,19 @@
         <v>93.735730602828497</v>
       </c>
       <c r="G40" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>18.386439347186197</v>
       </c>
       <c r="H40" s="1">
         <f t="shared" si="0"/>
         <v>6.2642693971715033</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I40" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>4</v>
       </c>
@@ -1727,15 +1889,19 @@
         <v>91.863099411614499</v>
       </c>
       <c r="G41" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>26.763298448097004</v>
       </c>
       <c r="H41" s="1">
         <f t="shared" si="0"/>
         <v>8.136900588385501</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I41" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>4</v>
       </c>
@@ -1755,15 +1921,19 @@
         <v>91.509898510780602</v>
       </c>
       <c r="G42" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>30.348620799958702</v>
       </c>
       <c r="H42" s="1">
         <f t="shared" si="0"/>
         <v>8.4901014892193984</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I42" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>4</v>
       </c>
@@ -1783,15 +1953,19 @@
         <v>91.503234342840301</v>
       </c>
       <c r="G43" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>32.8476837775573</v>
       </c>
       <c r="H43" s="1">
         <f t="shared" si="0"/>
         <v>8.496765657159699</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I43" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>4</v>
       </c>
@@ -1811,15 +1985,19 @@
         <v>91.676502709287107</v>
       </c>
       <c r="G44" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>33.387481380718604</v>
       </c>
       <c r="H44" s="1">
         <f t="shared" si="0"/>
         <v>8.3234972907128935</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I44" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>4</v>
       </c>
@@ -1839,15 +2017,19 @@
         <v>91.291758080202598</v>
       </c>
       <c r="G45" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>33.195997621901796</v>
       </c>
       <c r="H45" s="1">
         <f t="shared" si="0"/>
         <v>8.7082419197974019</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I45" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>4</v>
       </c>
@@ -1867,15 +2049,19 @@
         <v>91.316637640512894</v>
       </c>
       <c r="G46" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>33.407473884539392</v>
       </c>
       <c r="H46" s="1">
         <f t="shared" si="0"/>
         <v>8.6833623594871057</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I46" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>4</v>
       </c>
@@ -1895,15 +2081,19 @@
         <v>90.943444235858195</v>
       </c>
       <c r="G47" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>33.214213014271792</v>
       </c>
       <c r="H47" s="1">
         <f t="shared" si="0"/>
         <v>9.0565557641418053</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I47" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>4</v>
       </c>
@@ -1923,15 +2113,19 @@
         <v>90.470732589962196</v>
       </c>
       <c r="G48" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>33.141351444791596</v>
       </c>
       <c r="H48" s="1">
         <f t="shared" si="0"/>
         <v>9.5292674100378036</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I48" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>4</v>
       </c>
@@ -1951,15 +2145,19 @@
         <v>90.290355777712406</v>
       </c>
       <c r="G49" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>33.514100571583704</v>
       </c>
       <c r="H49" s="1">
         <f t="shared" si="0"/>
         <v>9.7096442222875936</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I49" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>4</v>
       </c>
@@ -1979,15 +2177,19 @@
         <v>90.103759075385</v>
       </c>
       <c r="G50" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>33.4141380524797</v>
       </c>
       <c r="H50" s="1">
         <f t="shared" si="0"/>
         <v>9.8962409246150003</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I50" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>4</v>
       </c>
@@ -1995,7 +2197,7 @@
         <v>22</v>
       </c>
       <c r="C51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D51" s="1">
         <v>56.679624770994899</v>
@@ -2007,15 +2209,19 @@
         <v>90.103759075385</v>
       </c>
       <c r="G51" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>33.424134304390101</v>
       </c>
       <c r="H51" s="1">
         <f t="shared" si="0"/>
         <v>9.8962409246150003</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I51" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>4</v>
       </c>
@@ -2023,7 +2229,7 @@
         <v>23</v>
       </c>
       <c r="C52" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D52" s="1">
         <v>56.509688488518201</v>
@@ -2035,15 +2241,19 @@
         <v>90.290355777712406</v>
       </c>
       <c r="G52" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>33.780667289194206</v>
       </c>
       <c r="H52" s="1">
         <f t="shared" si="0"/>
         <v>9.7096442222875936</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I52" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>4</v>
       </c>
@@ -2051,7 +2261,7 @@
         <v>24</v>
       </c>
       <c r="C53" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D53" s="1">
         <v>55.763301679208702</v>
@@ -2063,15 +2273,19 @@
         <v>90.290355777712406</v>
       </c>
       <c r="G53" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>34.527054098503704</v>
       </c>
       <c r="H53" s="1">
         <f t="shared" si="0"/>
         <v>9.7096442222875936</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I53" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>4</v>
       </c>
@@ -2079,7 +2293,7 @@
         <v>25</v>
       </c>
       <c r="C54" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D54" s="1">
         <v>54.445129260624697</v>
@@ -2091,15 +2305,19 @@
         <v>90.103759075385</v>
       </c>
       <c r="G54" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>35.658629814760303</v>
       </c>
       <c r="H54" s="1">
         <f t="shared" si="0"/>
         <v>9.8962409246150003</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I54" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>4</v>
       </c>
@@ -2107,7 +2325,7 @@
         <v>26</v>
       </c>
       <c r="C55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D55" s="1">
         <v>54.090595526202698</v>
@@ -2119,15 +2337,19 @@
         <v>90.103759075385</v>
       </c>
       <c r="G55" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>36.013163549182302</v>
       </c>
       <c r="H55" s="1">
         <f t="shared" si="0"/>
         <v>9.8962409246150003</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I55" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>4</v>
       </c>
@@ -2135,7 +2357,7 @@
         <v>27</v>
       </c>
       <c r="C56" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D56" s="1">
         <v>53.890670487994797</v>
@@ -2147,15 +2369,19 @@
         <v>89.917162373057593</v>
       </c>
       <c r="G56" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>36.026491885062796</v>
       </c>
       <c r="H56" s="1">
         <f t="shared" si="0"/>
         <v>10.082837626942407</v>
       </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I56" s="1">
+        <f t="shared" si="1"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>4</v>
       </c>
@@ -2163,7 +2389,7 @@
         <v>28</v>
       </c>
       <c r="C57" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D57" s="1">
         <v>53.150947846625598</v>

</xml_diff>